<commit_message>
import property by excel
</commit_message>
<xml_diff>
--- a/docs/SLMS2026_import_dot1_khoi_tao.xlsx
+++ b/docs/SLMS2026_import_dot1_khoi_tao.xlsx
@@ -8,7 +8,6 @@
     <sheet name="0. Danh_Muc_Tham_Khao" sheetId="3" r:id="rId3"/>
     <sheet name="1. Hop_Dong_Thue" sheetId="4" r:id="rId4"/>
     <sheet name="2. Thiet_Bi_Ban_Giao" sheetId="5" r:id="rId5"/>
-    <sheet name="3. Danh_Sach_Phong" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -402,14 +401,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A7"/>
   <cols>
-    <col min="1" max="1" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="52.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Hướng dẫn — Đợt 1: Khởi tạo nhà</v>
+        <v>Hướng dẫn — Đợt 1: Khởi tạo nhà (HĐ thuê từ chủ)</v>
       </c>
     </row>
     <row r="2">
@@ -419,70 +418,45 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Sheet "1. Hop_Dong_Thue": tạo Property + hợp đồng thuê inbound.</v>
+        <v>Sheet "1. Hop_Dong_Thue": tạo Property + hợp đồng thuê — LUÔN nguyên căn.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Sheet "2. Thiet_Bi_Ban_Giao" (tùy chọn): TB chủ nhà gốc bàn giao — CHỈ HIỂN THỊ.</v>
+        <v>Sheet "2. Thiet_Bi_Ban_Giao" (tùy chọn): TB chủ bàn giao — CHỈ HIỂN THỊ, không gắn phòng vận hành.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Sheet "3. Danh_Sach_Phong" (BẮT BUỘC nếu [THEO_PHONG]): liệt kê ĐỦ từng phòng = Tổng số phòng.</v>
+        <v>"Tổng số phòng" = đặc tính vật lý căn nhà thuê, không phải số phòng khai thác.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Sheet "0. Ma_Tran_Trường_Hop": bảng demo 6 trường hợp nghiệp vụ (BE không đọc).</v>
+        <v>Chia phòng / hình thức khai thác → quyết định ở file đợt 2.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Địa chỉ / Zone:</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>- Chỉ dùng Quận/Huyện + Tỉnh/Thành phố (2 cấp Zone). KHÔNG có cột Xã/Phường.</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>- Địa chỉ chi tiết ghi đủ số nhà, ngõ/đường.</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Tag trong Mô tả chi tiết (demo): [NGUYEN_CAN] hoặc [THEO_PHONG] — gợi ý cho BE khi code.</v>
+        <v>Xem sheet "0. Ma_Tran_Trường_Hop".</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F12"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="27.83203125" customWidth="1"/>
-    <col min="4" max="4" width="35.83203125" customWidth="1"/>
-    <col min="5" max="5" width="33.83203125" customWidth="1"/>
+    <col min="2" max="2" width="21.83203125" customWidth="1"/>
+    <col min="3" max="3" width="19.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
     <col min="6" max="6" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -491,16 +465,16 @@
         <v>Mã hợp đồng (demo)</v>
       </c>
       <c r="B1" t="str">
-        <v>Loại hình (BE)</v>
+        <v>Đợt 1 TB bàn giao</v>
       </c>
       <c r="C1" t="str">
-        <v>TB chủ bàn giao (đợt 1)</v>
+        <v>Đợt 2 hình thức</v>
       </c>
       <c r="D1" t="str">
-        <v>Có dòng cải tạo (đợt 2 sheet 1)</v>
+        <v>Đợt 2 cải tạo</v>
       </c>
       <c r="E1" t="str">
-        <v>Có TB mua mới (đợt 2 sheet 2)</v>
+        <v>Đợt 2 mua TB</v>
       </c>
       <c r="F1" t="str">
         <v>Diễn giải</v>
@@ -511,10 +485,10 @@
         <v>HD-WH-RENO-FURN</v>
       </c>
       <c r="B2" t="str">
-        <v>Nguyên căn</v>
+        <v>Có</v>
       </c>
       <c r="C2" t="str">
-        <v>Có</v>
+        <v>NGUYEN_CAN</v>
       </c>
       <c r="D2" t="str">
         <v>Có</v>
@@ -523,7 +497,7 @@
         <v>Có</v>
       </c>
       <c r="F2" t="str">
-        <v>Thuê nguyên căn — cải tạo + mua nội thất thêm (mặc định phổ biến)</v>
+        <v>Thuê nguyên căn — giữ nguyên căn sau cải tạo + mua nội thất</v>
       </c>
     </row>
     <row r="3">
@@ -531,19 +505,19 @@
         <v>HD-WH-NORENO-FURN</v>
       </c>
       <c r="B3" t="str">
-        <v>Nguyên căn</v>
+        <v>Có</v>
       </c>
       <c r="C3" t="str">
-        <v>Có</v>
+        <v>—</v>
       </c>
       <c r="D3" t="str">
-        <v>Không</v>
+        <v>—</v>
       </c>
       <c r="E3" t="str">
-        <v>Không</v>
+        <v>—</v>
       </c>
       <c r="F3" t="str">
-        <v>Thuê nguyên căn — không cải tạo, chỉ TB chủ bàn giao (đợt 1). Không có dòng đợt 2.</v>
+        <v>Không cải tạo — sau đợt 1 gửi Host luôn (không có file đợt 2)</v>
       </c>
     </row>
     <row r="4">
@@ -551,10 +525,10 @@
         <v>HD-WH-RENO-NOFURN</v>
       </c>
       <c r="B4" t="str">
-        <v>Nguyên căn</v>
+        <v>Không</v>
       </c>
       <c r="C4" t="str">
-        <v>Không</v>
+        <v>NGUYEN_CAN</v>
       </c>
       <c r="D4" t="str">
         <v>Có</v>
@@ -571,30 +545,30 @@
         <v>HD-WH-NORENO-NOFURN</v>
       </c>
       <c r="B5" t="str">
-        <v>Nguyên căn</v>
+        <v>Không</v>
       </c>
       <c r="C5" t="str">
-        <v>Không</v>
+        <v>—</v>
       </c>
       <c r="D5" t="str">
-        <v>Không</v>
+        <v>—</v>
       </c>
       <c r="E5" t="str">
-        <v>Không</v>
+        <v>—</v>
       </c>
       <c r="F5" t="str">
-        <v>Thuê nguyên căn — trống, không cải tạo không TB. Không có dòng đợt 2.</v>
+        <v>Nhà trống, không cải tạo — gửi Host sau đợt 1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>HD-ROOM-RENO-FURN</v>
+        <v>HD-WH-RENO-SPLIT</v>
       </c>
       <c r="B6" t="str">
-        <v>Theo phòng</v>
+        <v>Có</v>
       </c>
       <c r="C6" t="str">
-        <v>Có</v>
+        <v>THEO_PHONG (5 phòng)</v>
       </c>
       <c r="D6" t="str">
         <v>Có</v>
@@ -603,72 +577,42 @@
         <v>Có</v>
       </c>
       <c r="F6" t="str">
-        <v>Thuê theo phòng — mặc định có cải tạo + mua nội thất từng phòng</v>
+        <v>Thuê nguyên căn đợt 1 — đợt 2 chia 5 phòng khai thác + mua TB từng phòng</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>HD-ROOM-RENO-NOFURN</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Theo phòng</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Không</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Có</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Không</v>
-      </c>
-      <c r="F7" t="str">
-        <v>Thuê theo phòng — chỉ cải tạo, không mua TB mới</v>
+        <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v/>
+        <v>Quy tắc:</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Cách BE suy ra từ file đợt 2 (không cần cột Có cải tạo / Có nội thất):</v>
+        <v>- Đợt 1: luôn import nhà nguyên căn (HĐ thuê từ chủ). TB bàn giao chỉ ghi nhận, không gắn phòng.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>- Có cải tạo ⇔ tồn tại ≥1 dòng sheet "1. Hop_Dong_Cai_Tao" cho mã HĐ đó</v>
+        <v>- Đợt 2: sheet "1. Cau_Hinh_Khai_Thac" quyết định NGUYEN_CAN hay THEO_PHONG.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>- Có nội thất mua thêm ⇔ tồn tại ≥1 dòng sheet "2. Thiet_Bi_Mua_Moi" cho mã HĐ đó</v>
+        <v>- THEO_PHONG: sheet "2. Danh_Sach_Phong" bắt buộc đủ Số phòng khai thác.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>- TB chủ bàn giao ⇔ chỉ có ở đợt 1 sheet "2. Thiet_Bi_Ban_Giao" (hiển thị, không vận hành)</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>- Nguyên căn vs theo phòng: quyết định ở BE khi code đợt 1 (không có trong file đợt 2)</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v xml:space="preserve">  Gợi ý: prefix mã demo HD-WH-* = nguyên căn, HD-ROOM-* = theo phòng — hoặc rule nghiệp vụ BE chốt</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>- Nhà THEO_PHONG: sheet "3. Danh_Sach_Phong" BẮT BUỘC đủ số phòng = cột Tổng số phòng</v>
+        <v>- HD-*-NORENO-*: không có dòng trong file đợt 2.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F12"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -839,7 +783,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M6"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -935,7 +879,7 @@
         <v>2029-02-28</v>
       </c>
       <c r="M2" t="str">
-        <v>[NGUYEN_CAN] Biệt thự — cải tạo + mua nội thất thêm.</v>
+        <v>Biệt thự thuê nguyên căn — chờ cải tạo đợt 2.</v>
       </c>
     </row>
     <row r="3">
@@ -976,7 +920,7 @@
         <v>2031-04-30</v>
       </c>
       <c r="M3" t="str">
-        <v>[NGUYEN_CAN] Vào ở ngay — chỉ TB chủ bàn giao, không cải tạo.</v>
+        <v>Vào ở ngay — chỉ TB chủ bàn giao, không cải tạo.</v>
       </c>
     </row>
     <row r="4">
@@ -1017,7 +961,7 @@
         <v>2031-08-31</v>
       </c>
       <c r="M4" t="str">
-        <v>[NGUYEN_CAN] Cải tạo hoàn thiện, không mua TB mới.</v>
+        <v>Cải tạo hoàn thiện, không mua TB mới.</v>
       </c>
     </row>
     <row r="5">
@@ -1058,12 +1002,12 @@
         <v>2027-05-31</v>
       </c>
       <c r="M5" t="str">
-        <v>[NGUYEN_CAN] Nhà trống hoàn toàn, không cải tạo không TB.</v>
+        <v>Nhà trống hoàn toàn, không cải tạo.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>HD-ROOM-RENO-FURN</v>
+        <v>HD-WH-RENO-SPLIT</v>
       </c>
       <c r="B6" t="str">
         <v>Nhà trọ Bình Thạnh</v>
@@ -1084,7 +1028,7 @@
         <v>3</v>
       </c>
       <c r="H6">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="I6" t="str">
         <v>Lê Thị Hương</v>
@@ -1099,69 +1043,27 @@
         <v>2028-03-31</v>
       </c>
       <c r="M6" t="str">
-        <v>[THEO_PHONG] 10 phòng (101–110) — cải tạo + mua nội thất từng phòng.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>HD-ROOM-RENO-NOFURN</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Nhà trọ sinh viên Cầu Giấy</v>
-      </c>
-      <c r="C7" t="str">
-        <v>24 Xuân Thủy</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Cầu Giấy</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Hà Nội</v>
-      </c>
-      <c r="F7">
-        <v>110</v>
-      </c>
-      <c r="G7">
-        <v>4</v>
-      </c>
-      <c r="H7">
-        <v>10</v>
-      </c>
-      <c r="I7" t="str">
-        <v>Hoàng Văn Nam</v>
-      </c>
-      <c r="J7">
-        <v>380000000</v>
-      </c>
-      <c r="K7" t="str">
-        <v>2026-07-01</v>
-      </c>
-      <c r="L7" t="str">
-        <v>2029-06-30</v>
-      </c>
-      <c r="M7" t="str">
-        <v>[THEO_PHONG] 10 phòng — chỉ cải tạo, không mua TB.</v>
+        <v>Thuê nguyên căn từ chủ — đợt 2 sẽ chia phòng khai thác.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:G6"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
     <col min="3" max="3" width="18.83203125" customWidth="1"/>
     <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
-    <col min="6" max="6" width="23.83203125" customWidth="1"/>
+    <col min="5" max="5" width="23.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
     <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1175,18 +1077,15 @@
         <v>Mô tả chi tiết</v>
       </c>
       <c r="D1" t="str">
-        <v>Số phòng</v>
+        <v>Mô tả vị trí</v>
       </c>
       <c r="E1" t="str">
-        <v>Khu vực chung</v>
+        <v>Trạng thái thiết bị</v>
       </c>
       <c r="F1" t="str">
-        <v>Trạng thái thiết bị</v>
+        <v>Số lượng</v>
       </c>
       <c r="G1" t="str">
-        <v>Số lượng</v>
-      </c>
-      <c r="H1" t="str">
         <v>Ghi chú</v>
       </c>
     </row>
@@ -1198,21 +1097,18 @@
         <v>Điều hòa</v>
       </c>
       <c r="C2" t="str">
-        <v>Máy lạnh 2HP tầng 1</v>
+        <v>Máy lạnh 2HP cũ</v>
       </c>
       <c r="D2" t="str">
-        <v>101</v>
+        <v>Tầng 1, phòng khách</v>
       </c>
       <c r="E2" t="str">
-        <v/>
-      </c>
-      <c r="F2" t="str">
         <v>GOOD</v>
       </c>
-      <c r="G2">
+      <c r="F2">
         <v>2</v>
       </c>
-      <c r="H2" t="str">
+      <c r="G2" t="str">
         <v>Chủ bàn giao</v>
       </c>
     </row>
@@ -1224,21 +1120,18 @@
         <v>Tủ lạnh</v>
       </c>
       <c r="C3" t="str">
-        <v>Tủ 250L cũ</v>
+        <v>Tủ 250L</v>
       </c>
       <c r="D3" t="str">
-        <v/>
+        <v>Nhà bếp</v>
       </c>
       <c r="E3" t="str">
-        <v>KITCHEN</v>
-      </c>
-      <c r="F3" t="str">
         <v>GOOD</v>
       </c>
-      <c r="G3">
+      <c r="F3">
         <v>1</v>
       </c>
-      <c r="H3" t="str">
+      <c r="G3" t="str">
         <v/>
       </c>
     </row>
@@ -1250,22 +1143,19 @@
         <v>Điều hòa</v>
       </c>
       <c r="C4" t="str">
-        <v>3 máy lạnh các phòng</v>
+        <v>3 máy lạnh</v>
       </c>
       <c r="D4" t="str">
-        <v>101</v>
+        <v>Các phòng trong nhà</v>
       </c>
       <c r="E4" t="str">
+        <v>GOOD</v>
+      </c>
+      <c r="F4">
+        <v>3</v>
+      </c>
+      <c r="G4" t="str">
         <v/>
-      </c>
-      <c r="F4" t="str">
-        <v>GOOD</v>
-      </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-      <c r="H4" t="str">
-        <v>Phòng 101</v>
       </c>
     </row>
     <row r="5">
@@ -1273,691 +1163,50 @@
         <v>HD-WH-NORENO-FURN</v>
       </c>
       <c r="B5" t="str">
-        <v>Điều hòa</v>
+        <v>Máy giặt</v>
       </c>
       <c r="C5" t="str">
+        <v>Máy giặt sân sau</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Sân sau</v>
+      </c>
+      <c r="E5" t="str">
+        <v>GOOD</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5" t="str">
         <v/>
-      </c>
-      <c r="D5" t="str">
-        <v>102</v>
-      </c>
-      <c r="E5" t="str">
-        <v/>
-      </c>
-      <c r="F5" t="str">
-        <v>GOOD</v>
-      </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-      <c r="H5" t="str">
-        <v>Phòng 102</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>HD-WH-NORENO-FURN</v>
+        <v>HD-WH-RENO-SPLIT</v>
       </c>
       <c r="B6" t="str">
-        <v>Máy giặt</v>
+        <v>Quạt</v>
       </c>
       <c r="C6" t="str">
-        <v>Máy giặt sân sau</v>
+        <v>Quạt trần cũ</v>
       </c>
       <c r="D6" t="str">
-        <v/>
+        <v>Toàn nhà</v>
       </c>
       <c r="E6" t="str">
-        <v>GARAGE</v>
-      </c>
-      <c r="F6" t="str">
         <v>GOOD</v>
       </c>
-      <c r="G6">
-        <v>1</v>
-      </c>
-      <c r="H6" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>HD-ROOM-RENO-FURN</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Điều hòa</v>
-      </c>
-      <c r="C7" t="str">
-        <v>TB chủ bàn giao phòng 101</v>
-      </c>
-      <c r="D7" t="str">
-        <v>101</v>
-      </c>
-      <c r="E7" t="str">
-        <v/>
-      </c>
-      <c r="F7" t="str">
-        <v>GOOD</v>
-      </c>
-      <c r="G7">
-        <v>1</v>
-      </c>
-      <c r="H7" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>HD-ROOM-RENO-FURN</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Điều hòa</v>
-      </c>
-      <c r="C8" t="str">
-        <v>TB chủ bàn giao phòng 102</v>
-      </c>
-      <c r="D8" t="str">
-        <v>102</v>
-      </c>
-      <c r="E8" t="str">
-        <v/>
-      </c>
-      <c r="F8" t="str">
-        <v>GOOD</v>
-      </c>
-      <c r="G8">
-        <v>1</v>
-      </c>
-      <c r="H8" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>HD-ROOM-RENO-FURN</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Điều hòa</v>
-      </c>
-      <c r="C9" t="str">
-        <v>TB chủ bàn giao phòng 103</v>
-      </c>
-      <c r="D9" t="str">
-        <v>103</v>
-      </c>
-      <c r="E9" t="str">
-        <v/>
-      </c>
-      <c r="F9" t="str">
-        <v>GOOD</v>
-      </c>
-      <c r="G9">
-        <v>1</v>
-      </c>
-      <c r="H9" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>HD-ROOM-RENO-FURN</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Điều hòa</v>
-      </c>
-      <c r="C10" t="str">
-        <v>TB chủ bàn giao phòng 104</v>
-      </c>
-      <c r="D10" t="str">
-        <v>104</v>
-      </c>
-      <c r="E10" t="str">
-        <v/>
-      </c>
-      <c r="F10" t="str">
-        <v>GOOD</v>
-      </c>
-      <c r="G10">
-        <v>1</v>
-      </c>
-      <c r="H10" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>HD-ROOM-RENO-FURN</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Điều hòa</v>
-      </c>
-      <c r="C11" t="str">
-        <v>TB chủ bàn giao phòng 105</v>
-      </c>
-      <c r="D11" t="str">
-        <v>105</v>
-      </c>
-      <c r="E11" t="str">
-        <v/>
-      </c>
-      <c r="F11" t="str">
-        <v>GOOD</v>
-      </c>
-      <c r="G11">
-        <v>1</v>
-      </c>
-      <c r="H11" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>HD-ROOM-RENO-FURN</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Điều hòa</v>
-      </c>
-      <c r="C12" t="str">
-        <v>TB chủ bàn giao phòng 106</v>
-      </c>
-      <c r="D12" t="str">
-        <v>106</v>
-      </c>
-      <c r="E12" t="str">
-        <v/>
-      </c>
-      <c r="F12" t="str">
-        <v>GOOD</v>
-      </c>
-      <c r="G12">
-        <v>1</v>
-      </c>
-      <c r="H12" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>HD-ROOM-RENO-FURN</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Điều hòa</v>
-      </c>
-      <c r="C13" t="str">
-        <v>TB chủ bàn giao phòng 107</v>
-      </c>
-      <c r="D13" t="str">
-        <v>107</v>
-      </c>
-      <c r="E13" t="str">
-        <v/>
-      </c>
-      <c r="F13" t="str">
-        <v>GOOD</v>
-      </c>
-      <c r="G13">
-        <v>1</v>
-      </c>
-      <c r="H13" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>HD-ROOM-RENO-FURN</v>
-      </c>
-      <c r="B14" t="str">
-        <v>Điều hòa</v>
-      </c>
-      <c r="C14" t="str">
-        <v>TB chủ bàn giao phòng 108</v>
-      </c>
-      <c r="D14" t="str">
-        <v>108</v>
-      </c>
-      <c r="E14" t="str">
-        <v/>
-      </c>
-      <c r="F14" t="str">
-        <v>GOOD</v>
-      </c>
-      <c r="G14">
-        <v>1</v>
-      </c>
-      <c r="H14" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>HD-ROOM-RENO-FURN</v>
-      </c>
-      <c r="B15" t="str">
-        <v>Điều hòa</v>
-      </c>
-      <c r="C15" t="str">
-        <v>TB chủ bàn giao phòng 109</v>
-      </c>
-      <c r="D15" t="str">
-        <v>109</v>
-      </c>
-      <c r="E15" t="str">
-        <v/>
-      </c>
-      <c r="F15" t="str">
-        <v>GOOD</v>
-      </c>
-      <c r="G15">
-        <v>1</v>
-      </c>
-      <c r="H15" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>HD-ROOM-RENO-FURN</v>
-      </c>
-      <c r="B16" t="str">
-        <v>Điều hòa</v>
-      </c>
-      <c r="C16" t="str">
-        <v>TB chủ bàn giao phòng 110</v>
-      </c>
-      <c r="D16" t="str">
-        <v>110</v>
-      </c>
-      <c r="E16" t="str">
-        <v/>
-      </c>
-      <c r="F16" t="str">
-        <v>GOOD</v>
-      </c>
-      <c r="G16">
-        <v>1</v>
-      </c>
-      <c r="H16" t="str">
-        <v/>
+      <c r="F6">
+        <v>5</v>
+      </c>
+      <c r="G6" t="str">
+        <v>TB chủ bàn giao trước cải tạo</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H16"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E21"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="24.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Mã hợp đồng thuê</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Số phòng</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Tầng</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Diện tích phòng (m²)</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Ghi chú</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>HD-ROOM-RENO-FURN</v>
-      </c>
-      <c r="B2" t="str">
-        <v>101</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>12</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Phòng 101</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>HD-ROOM-RENO-FURN</v>
-      </c>
-      <c r="B3" t="str">
-        <v>102</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>12</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Phòng 102</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>HD-ROOM-RENO-FURN</v>
-      </c>
-      <c r="B4" t="str">
-        <v>103</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="D4">
-        <v>12</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Phòng 103</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>HD-ROOM-RENO-FURN</v>
-      </c>
-      <c r="B5" t="str">
-        <v>104</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>12</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Phòng 104</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>HD-ROOM-RENO-FURN</v>
-      </c>
-      <c r="B6" t="str">
-        <v>105</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-      <c r="D6">
-        <v>12</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Phòng 105</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>HD-ROOM-RENO-FURN</v>
-      </c>
-      <c r="B7" t="str">
-        <v>106</v>
-      </c>
-      <c r="C7">
-        <v>1</v>
-      </c>
-      <c r="D7">
-        <v>12</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Phòng 106</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>HD-ROOM-RENO-FURN</v>
-      </c>
-      <c r="B8" t="str">
-        <v>107</v>
-      </c>
-      <c r="C8">
-        <v>1</v>
-      </c>
-      <c r="D8">
-        <v>12</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Phòng 107</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>HD-ROOM-RENO-FURN</v>
-      </c>
-      <c r="B9" t="str">
-        <v>108</v>
-      </c>
-      <c r="C9">
-        <v>1</v>
-      </c>
-      <c r="D9">
-        <v>12</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Phòng 108</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>HD-ROOM-RENO-FURN</v>
-      </c>
-      <c r="B10" t="str">
-        <v>109</v>
-      </c>
-      <c r="C10">
-        <v>1</v>
-      </c>
-      <c r="D10">
-        <v>12</v>
-      </c>
-      <c r="E10" t="str">
-        <v>Phòng 109</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>HD-ROOM-RENO-FURN</v>
-      </c>
-      <c r="B11" t="str">
-        <v>110</v>
-      </c>
-      <c r="C11">
-        <v>1</v>
-      </c>
-      <c r="D11">
-        <v>12</v>
-      </c>
-      <c r="E11" t="str">
-        <v>Phòng 110</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>HD-ROOM-RENO-NOFURN</v>
-      </c>
-      <c r="B12" t="str">
-        <v>101</v>
-      </c>
-      <c r="C12">
-        <v>1</v>
-      </c>
-      <c r="D12">
-        <v>11</v>
-      </c>
-      <c r="E12" t="str">
-        <v>Phòng 101</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>HD-ROOM-RENO-NOFURN</v>
-      </c>
-      <c r="B13" t="str">
-        <v>102</v>
-      </c>
-      <c r="C13">
-        <v>1</v>
-      </c>
-      <c r="D13">
-        <v>11</v>
-      </c>
-      <c r="E13" t="str">
-        <v>Phòng 102</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>HD-ROOM-RENO-NOFURN</v>
-      </c>
-      <c r="B14" t="str">
-        <v>103</v>
-      </c>
-      <c r="C14">
-        <v>1</v>
-      </c>
-      <c r="D14">
-        <v>11</v>
-      </c>
-      <c r="E14" t="str">
-        <v>Phòng 103</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>HD-ROOM-RENO-NOFURN</v>
-      </c>
-      <c r="B15" t="str">
-        <v>104</v>
-      </c>
-      <c r="C15">
-        <v>1</v>
-      </c>
-      <c r="D15">
-        <v>11</v>
-      </c>
-      <c r="E15" t="str">
-        <v>Phòng 104</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>HD-ROOM-RENO-NOFURN</v>
-      </c>
-      <c r="B16" t="str">
-        <v>105</v>
-      </c>
-      <c r="C16">
-        <v>1</v>
-      </c>
-      <c r="D16">
-        <v>11</v>
-      </c>
-      <c r="E16" t="str">
-        <v>Phòng 105</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>HD-ROOM-RENO-NOFURN</v>
-      </c>
-      <c r="B17" t="str">
-        <v>106</v>
-      </c>
-      <c r="C17">
-        <v>1</v>
-      </c>
-      <c r="D17">
-        <v>11</v>
-      </c>
-      <c r="E17" t="str">
-        <v>Phòng 106</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>HD-ROOM-RENO-NOFURN</v>
-      </c>
-      <c r="B18" t="str">
-        <v>107</v>
-      </c>
-      <c r="C18">
-        <v>1</v>
-      </c>
-      <c r="D18">
-        <v>11</v>
-      </c>
-      <c r="E18" t="str">
-        <v>Phòng 107</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>HD-ROOM-RENO-NOFURN</v>
-      </c>
-      <c r="B19" t="str">
-        <v>108</v>
-      </c>
-      <c r="C19">
-        <v>1</v>
-      </c>
-      <c r="D19">
-        <v>11</v>
-      </c>
-      <c r="E19" t="str">
-        <v>Phòng 108</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>HD-ROOM-RENO-NOFURN</v>
-      </c>
-      <c r="B20" t="str">
-        <v>109</v>
-      </c>
-      <c r="C20">
-        <v>1</v>
-      </c>
-      <c r="D20">
-        <v>11</v>
-      </c>
-      <c r="E20" t="str">
-        <v>Phòng 109</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>HD-ROOM-RENO-NOFURN</v>
-      </c>
-      <c r="B21" t="str">
-        <v>110</v>
-      </c>
-      <c r="C21">
-        <v>1</v>
-      </c>
-      <c r="D21">
-        <v>11</v>
-      </c>
-      <c r="E21" t="str">
-        <v>Phòng 110</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add length and width of room and property
</commit_message>
<xml_diff>
--- a/docs/SLMS2026_import_dot1_khoi_tao.xlsx
+++ b/docs/SLMS2026_import_dot1_khoi_tao.xlsx
@@ -988,7 +988,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M16"/>
+  <dimension ref="A1:O16"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -1003,6 +1003,8 @@
     <col min="11" max="11" width="18.83203125" customWidth="1"/>
     <col min="12" max="12" width="18.83203125" customWidth="1"/>
     <col min="13" max="13" width="18.83203125" customWidth="1"/>
+    <col min="14" max="14" width="18.83203125" customWidth="1"/>
+    <col min="15" max="15" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1025,24 +1027,30 @@
         <v>Diện tích (m²)</v>
       </c>
       <c r="G1" t="str">
+        <v>Chiều dài (m)</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Chiều rộng (m)</v>
+      </c>
+      <c r="I1" t="str">
         <v>Tổng số tầng</v>
       </c>
-      <c r="H1" t="str">
+      <c r="J1" t="str">
         <v>Tổng số phòng</v>
       </c>
-      <c r="I1" t="str">
+      <c r="K1" t="str">
         <v>Tên chủ nhà</v>
       </c>
-      <c r="J1" t="str">
+      <c r="L1" t="str">
         <v>Tổng tiền thuê</v>
       </c>
-      <c r="K1" t="str">
+      <c r="M1" t="str">
         <v>Ngày bắt đầu</v>
       </c>
-      <c r="L1" t="str">
+      <c r="N1" t="str">
         <v>Ngày kết thúc</v>
       </c>
-      <c r="M1" t="str">
+      <c r="O1" t="str">
         <v>Mô tả chi tiết</v>
       </c>
     </row>
@@ -1066,24 +1074,30 @@
         <v>180</v>
       </c>
       <c r="G2">
+        <v>15.9</v>
+      </c>
+      <c r="H2">
+        <v>11.3</v>
+      </c>
+      <c r="I2">
         <v>2</v>
       </c>
-      <c r="H2">
+      <c r="J2">
         <v>5</v>
       </c>
-      <c r="I2" t="str">
+      <c r="K2" t="str">
         <v>Trần Minh Tuấn</v>
       </c>
-      <c r="J2">
+      <c r="L2">
         <v>450000000</v>
       </c>
-      <c r="K2" t="str">
+      <c r="M2" t="str">
         <v>2026-03-01</v>
       </c>
-      <c r="L2" t="str">
+      <c r="N2" t="str">
         <v>2029-02-28</v>
       </c>
-      <c r="M2" t="str">
+      <c r="O2" t="str">
         <v>Biệt thự thuê nguyên căn — chờ cải tạo đợt 2.</v>
       </c>
     </row>
@@ -1107,24 +1121,30 @@
         <v>95</v>
       </c>
       <c r="G3">
+        <v>11.5</v>
+      </c>
+      <c r="H3">
+        <v>8.3</v>
+      </c>
+      <c r="I3">
         <v>2</v>
       </c>
-      <c r="H3">
+      <c r="J3">
         <v>4</v>
       </c>
-      <c r="I3" t="str">
+      <c r="K3" t="str">
         <v>Phạm Văn Đức</v>
       </c>
-      <c r="J3">
+      <c r="L3">
         <v>280000000</v>
       </c>
-      <c r="K3" t="str">
+      <c r="M3" t="str">
         <v>2026-05-01</v>
       </c>
-      <c r="L3" t="str">
+      <c r="N3" t="str">
         <v>2031-04-30</v>
       </c>
-      <c r="M3" t="str">
+      <c r="O3" t="str">
         <v>Vào ở ngay — chỉ TB chủ bàn giao, không cải tạo.</v>
       </c>
     </row>
@@ -1148,24 +1168,30 @@
         <v>200</v>
       </c>
       <c r="G4">
+        <v>16.7</v>
+      </c>
+      <c r="H4">
+        <v>12</v>
+      </c>
+      <c r="I4">
         <v>1</v>
       </c>
-      <c r="H4">
+      <c r="J4">
         <v>4</v>
       </c>
-      <c r="I4" t="str">
+      <c r="K4" t="str">
         <v>Đặng Quốc Bảo</v>
       </c>
-      <c r="J4">
+      <c r="L4">
         <v>550000000</v>
       </c>
-      <c r="K4" t="str">
+      <c r="M4" t="str">
         <v>2026-09-01</v>
       </c>
-      <c r="L4" t="str">
+      <c r="N4" t="str">
         <v>2031-08-31</v>
       </c>
-      <c r="M4" t="str">
+      <c r="O4" t="str">
         <v>Cải tạo hoàn thiện, không mua TB mới.</v>
       </c>
     </row>
@@ -1189,24 +1215,30 @@
         <v>55</v>
       </c>
       <c r="G5">
+        <v>8.8</v>
+      </c>
+      <c r="H5">
+        <v>6.2</v>
+      </c>
+      <c r="I5">
         <v>1</v>
       </c>
-      <c r="H5">
+      <c r="J5">
         <v>1</v>
       </c>
-      <c r="I5" t="str">
+      <c r="K5" t="str">
         <v>Nguyễn Thu Hà</v>
       </c>
-      <c r="J5">
+      <c r="L5">
         <v>180000000</v>
       </c>
-      <c r="K5" t="str">
+      <c r="M5" t="str">
         <v>2026-06-01</v>
       </c>
-      <c r="L5" t="str">
+      <c r="N5" t="str">
         <v>2027-05-31</v>
       </c>
-      <c r="M5" t="str">
+      <c r="O5" t="str">
         <v>Nhà trống hoàn toàn, không cải tạo.</v>
       </c>
     </row>
@@ -1230,24 +1262,30 @@
         <v>120</v>
       </c>
       <c r="G6">
+        <v>13</v>
+      </c>
+      <c r="H6">
+        <v>9.2</v>
+      </c>
+      <c r="I6">
         <v>3</v>
       </c>
-      <c r="H6">
+      <c r="J6">
         <v>8</v>
       </c>
-      <c r="I6" t="str">
+      <c r="K6" t="str">
         <v>Lê Thị Hương</v>
       </c>
-      <c r="J6">
+      <c r="L6">
         <v>320000000</v>
       </c>
-      <c r="K6" t="str">
+      <c r="M6" t="str">
         <v>2026-04-01</v>
       </c>
-      <c r="L6" t="str">
+      <c r="N6" t="str">
         <v>2028-03-31</v>
       </c>
-      <c r="M6" t="str">
+      <c r="O6" t="str">
         <v>Thuê nguyên căn từ chủ — đợt 2 chia 5 phòng khai thác.</v>
       </c>
     </row>
@@ -1271,24 +1309,30 @@
         <v>160</v>
       </c>
       <c r="G7">
+        <v>15</v>
+      </c>
+      <c r="H7">
+        <v>10.7</v>
+      </c>
+      <c r="I7">
         <v>4</v>
       </c>
-      <c r="H7">
+      <c r="J7">
         <v>10</v>
       </c>
-      <c r="I7" t="str">
+      <c r="K7" t="str">
         <v>Võ Minh Khang</v>
       </c>
-      <c r="J7">
+      <c r="L7">
         <v>380000000</v>
       </c>
-      <c r="K7" t="str">
+      <c r="M7" t="str">
         <v>2026-02-01</v>
       </c>
-      <c r="L7" t="str">
+      <c r="N7" t="str">
         <v>2029-01-31</v>
       </c>
-      <c r="M7" t="str">
+      <c r="O7" t="str">
         <v>Nhà trọ lớn — chia 8 phòng khai thác.</v>
       </c>
     </row>
@@ -1312,24 +1356,30 @@
         <v>75</v>
       </c>
       <c r="G8">
+        <v>10.2</v>
+      </c>
+      <c r="H8">
+        <v>7.4</v>
+      </c>
+      <c r="I8">
         <v>2</v>
       </c>
-      <c r="H8">
+      <c r="J8">
         <v>3</v>
       </c>
-      <c r="I8" t="str">
+      <c r="K8" t="str">
         <v>Hoàng Thị Lan</v>
       </c>
-      <c r="J8">
+      <c r="L8">
         <v>220000000</v>
       </c>
-      <c r="K8" t="str">
+      <c r="M8" t="str">
         <v>2026-07-01</v>
       </c>
-      <c r="L8" t="str">
+      <c r="N8" t="str">
         <v>2028-06-30</v>
       </c>
-      <c r="M8" t="str">
+      <c r="O8" t="str">
         <v>Nhà nhỏ chia 3 phòng — không TB bàn giao.</v>
       </c>
     </row>
@@ -1353,24 +1403,30 @@
         <v>68</v>
       </c>
       <c r="G9">
+        <v>9.8</v>
+      </c>
+      <c r="H9">
+        <v>6.9</v>
+      </c>
+      <c r="I9">
         <v>1</v>
       </c>
-      <c r="H9">
+      <c r="J9">
         <v>2</v>
       </c>
-      <c r="I9" t="str">
+      <c r="K9" t="str">
         <v>Bùi Văn Nam</v>
       </c>
-      <c r="J9">
+      <c r="L9">
         <v>195000000</v>
       </c>
-      <c r="K9" t="str">
+      <c r="M9" t="str">
         <v>2026-08-01</v>
       </c>
-      <c r="L9" t="str">
+      <c r="N9" t="str">
         <v>2027-07-31</v>
       </c>
-      <c r="M9" t="str">
+      <c r="O9" t="str">
         <v>Không cải tạo lớn — chỉ mua TB mới nguyên căn.</v>
       </c>
     </row>
@@ -1394,24 +1450,30 @@
         <v>90</v>
       </c>
       <c r="G10">
+        <v>11.2</v>
+      </c>
+      <c r="H10">
+        <v>8</v>
+      </c>
+      <c r="I10">
         <v>3</v>
       </c>
-      <c r="H10">
+      <c r="J10">
         <v>4</v>
       </c>
-      <c r="I10" t="str">
+      <c r="K10" t="str">
         <v>Nguyễn Văn Hùng</v>
       </c>
-      <c r="J10">
+      <c r="L10">
         <v>240000000</v>
       </c>
-      <c r="K10" t="str">
+      <c r="M10" t="str">
         <v>2026-04-15</v>
       </c>
-      <c r="L10" t="str">
+      <c r="N10" t="str">
         <v>2029-04-14</v>
       </c>
-      <c r="M10" t="str">
+      <c r="O10" t="str">
         <v>Hà Nội — cải tạo tối thiểu 1 hạng mục.</v>
       </c>
     </row>
@@ -1435,24 +1497,30 @@
         <v>110</v>
       </c>
       <c r="G11">
+        <v>12.4</v>
+      </c>
+      <c r="H11">
+        <v>8.9</v>
+      </c>
+      <c r="I11">
         <v>2</v>
       </c>
-      <c r="H11">
+      <c r="J11">
         <v>3</v>
       </c>
-      <c r="I11" t="str">
+      <c r="K11" t="str">
         <v>Trịnh Quốc Anh</v>
       </c>
-      <c r="J11">
+      <c r="L11">
         <v>420000000</v>
       </c>
-      <c r="K11" t="str">
+      <c r="M11" t="str">
         <v>2026-10-01</v>
       </c>
-      <c r="L11" t="str">
+      <c r="N11" t="str">
         <v>2030-09-30</v>
       </c>
-      <c r="M11" t="str">
+      <c r="O11" t="str">
         <v>TB bàn giao nhiều trạng thái hỏng — không cải tạo.</v>
       </c>
     </row>
@@ -1476,24 +1544,30 @@
         <v>140</v>
       </c>
       <c r="G12">
+        <v>14</v>
+      </c>
+      <c r="H12">
+        <v>10</v>
+      </c>
+      <c r="I12">
         <v>2</v>
       </c>
-      <c r="H12">
+      <c r="J12">
         <v>6</v>
       </c>
-      <c r="I12" t="str">
+      <c r="K12" t="str">
         <v>Lý Thanh Tùng</v>
       </c>
-      <c r="J12">
+      <c r="L12">
         <v>360000000</v>
       </c>
-      <c r="K12" t="str">
+      <c r="M12" t="str">
         <v>2026-05-15</v>
       </c>
-      <c r="L12" t="str">
+      <c r="N12" t="str">
         <v>2030-05-14</v>
       </c>
-      <c r="M12" t="str">
+      <c r="O12" t="str">
         <v>Cải tạo kết cấu + nội thất nguyên căn.</v>
       </c>
     </row>
@@ -1517,24 +1591,30 @@
         <v>220</v>
       </c>
       <c r="G13">
+        <v>17.5</v>
+      </c>
+      <c r="H13">
+        <v>12.6</v>
+      </c>
+      <c r="I13">
         <v>4</v>
       </c>
-      <c r="H13">
+      <c r="J13">
         <v>14</v>
       </c>
-      <c r="I13" t="str">
+      <c r="K13" t="str">
         <v>Đỗ Thị Mai</v>
       </c>
-      <c r="J13">
+      <c r="L13">
         <v>520000000</v>
       </c>
-      <c r="K13" t="str">
+      <c r="M13" t="str">
         <v>2026-01-01</v>
       </c>
-      <c r="L13" t="str">
+      <c r="N13" t="str">
         <v>2030-12-31</v>
       </c>
-      <c r="M13" t="str">
+      <c r="O13" t="str">
         <v>Ký túc xá mini — 12 phòng khai thác.</v>
       </c>
     </row>
@@ -1558,24 +1638,30 @@
         <v>80</v>
       </c>
       <c r="G14">
+        <v>10.6</v>
+      </c>
+      <c r="H14">
+        <v>7.5</v>
+      </c>
+      <c r="I14">
         <v>2</v>
       </c>
-      <c r="H14">
+      <c r="J14">
         <v>3</v>
       </c>
-      <c r="I14" t="str">
+      <c r="K14" t="str">
         <v>Phan Minh Đức</v>
       </c>
-      <c r="J14">
+      <c r="L14">
         <v>200000000</v>
       </c>
-      <c r="K14" t="str">
+      <c r="M14" t="str">
         <v>2026-11-01</v>
       </c>
-      <c r="L14" t="str">
+      <c r="N14" t="str">
         <v>2028-10-31</v>
       </c>
-      <c r="M14" t="str">
+      <c r="O14" t="str">
         <v>Hà Nội — vào ở ngay, không cải tạo.</v>
       </c>
     </row>
@@ -1599,24 +1685,30 @@
         <v>250</v>
       </c>
       <c r="G15">
+        <v>18.7</v>
+      </c>
+      <c r="H15">
+        <v>13.4</v>
+      </c>
+      <c r="I15">
         <v>3</v>
       </c>
-      <c r="H15">
+      <c r="J15">
         <v>7</v>
       </c>
-      <c r="I15" t="str">
+      <c r="K15" t="str">
         <v>Vũ Thị Hồng</v>
       </c>
-      <c r="J15">
+      <c r="L15">
         <v>600000000</v>
       </c>
-      <c r="K15" t="str">
+      <c r="M15" t="str">
         <v>2026-03-15</v>
       </c>
-      <c r="L15" t="str">
+      <c r="N15" t="str">
         <v>2031-03-14</v>
       </c>
-      <c r="M15" t="str">
+      <c r="O15" t="str">
         <v>Biệt thự Hà Nội — cải tạo + mua TB cao cấp.</v>
       </c>
     </row>
@@ -1640,30 +1732,36 @@
         <v>100</v>
       </c>
       <c r="G16">
+        <v>11.8</v>
+      </c>
+      <c r="H16">
+        <v>8.5</v>
+      </c>
+      <c r="I16">
         <v>3</v>
       </c>
-      <c r="H16">
+      <c r="J16">
         <v>6</v>
       </c>
-      <c r="I16" t="str">
+      <c r="K16" t="str">
         <v>Trần Văn Phúc</v>
       </c>
-      <c r="J16">
+      <c r="L16">
         <v>270000000</v>
       </c>
-      <c r="K16" t="str">
+      <c r="M16" t="str">
         <v>2026-06-01</v>
       </c>
-      <c r="L16" t="str">
+      <c r="N16" t="str">
         <v>2028-05-31</v>
       </c>
-      <c r="M16" t="str">
+      <c r="O16" t="str">
         <v>Hà Nội — chia 5 phòng khai thác.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O16"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(lead wishlist): add feature
</commit_message>
<xml_diff>
--- a/docs/SLMS2026_import_dot1_khoi_tao.xlsx
+++ b/docs/SLMS2026_import_dot1_khoi_tao.xlsx
@@ -631,13 +631,13 @@
         <v>NGUYEN_CAN</v>
       </c>
       <c r="D9" t="str">
-        <v>Không</v>
+        <v>Có</v>
       </c>
       <c r="E9" t="str">
         <v>Có</v>
       </c>
       <c r="F9" t="str">
-        <v>NGUYEN_CAN — không dòng cải tạo, chỉ mua TB</v>
+        <v>NGUYEN_CAN — 1 hạng mục cải tạo nhẹ + mua TB</v>
       </c>
     </row>
     <row r="10">
@@ -1427,7 +1427,7 @@
         <v>2027-07-31</v>
       </c>
       <c r="O9" t="str">
-        <v>Không cải tạo lớn — chỉ mua TB mới nguyên căn.</v>
+        <v>Cải tạo nhẹ — chủ yếu mua TB mới nguyên căn.</v>
       </c>
     </row>
     <row r="10">

</xml_diff>